<commit_message>
Project 7/V2 - Revised data and result
</commit_message>
<xml_diff>
--- a/Project-7 ---/V2/Data/cancer_data_imputed.Farhana.xlsx
+++ b/Project-7 ---/V2/Data/cancer_data_imputed.Farhana.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Ibrahim\Statistical-Analysis\Project-7 ---\V2\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Freelance\Statistical-Analysis\Project-7 ---\V3\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD247EBD-B15C-4ECC-960E-B881B321C7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FABA3EAE-3466-4B47-AD2C-0366604A3AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9765" yWindow="60" windowWidth="17250" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -802,16 +802,16 @@
     <t xml:space="preserve">&gt;3 site </t>
   </si>
   <si>
-    <t>&gt;3site</t>
-  </si>
-  <si>
     <t xml:space="preserve">1 site </t>
   </si>
   <si>
     <t>negative</t>
   </si>
   <si>
-    <t>BCS</t>
+    <t>Biopsy</t>
+  </si>
+  <si>
+    <t>No Surgery</t>
   </si>
 </sst>
 </file>
@@ -1154,6 +1154,7 @@
   <dimension ref="A1:DA136"/>
   <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="43" max="43" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="71" max="71" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="72" max="72" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="83" max="83" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -1589,7 +1590,7 @@
         <v>105</v>
       </c>
       <c r="AT2" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU2" t="s">
         <v>118</v>
@@ -1882,7 +1883,7 @@
         <v>111</v>
       </c>
       <c r="AT3" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU3" t="s">
         <v>118</v>
@@ -2166,7 +2167,7 @@
         <v>107</v>
       </c>
       <c r="AT4" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU4" t="s">
         <v>118</v>
@@ -2447,19 +2448,19 @@
         <v>157</v>
       </c>
       <c r="AR5" t="s">
-        <v>260</v>
+        <v>147</v>
       </c>
       <c r="AS5" t="s">
         <v>107</v>
       </c>
       <c r="AT5" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU5" t="s">
         <v>118</v>
       </c>
       <c r="AV5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AW5" t="s">
         <v>120</v>
@@ -2749,7 +2750,7 @@
         <v>107</v>
       </c>
       <c r="AT6" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="AU6" t="s">
         <v>118</v>
@@ -3030,7 +3031,7 @@
         <v>107</v>
       </c>
       <c r="AT7" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU7" t="s">
         <v>118</v>
@@ -3302,13 +3303,13 @@
         <v>169</v>
       </c>
       <c r="AR8" t="s">
-        <v>259</v>
+        <v>147</v>
       </c>
       <c r="AS8" t="s">
         <v>105</v>
       </c>
       <c r="AT8" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU8" t="s">
         <v>118</v>
@@ -3595,7 +3596,7 @@
         <v>107</v>
       </c>
       <c r="AT9" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU9" t="s">
         <v>118</v>
@@ -3888,7 +3889,7 @@
         <v>107</v>
       </c>
       <c r="AT10" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU10" t="s">
         <v>118</v>
@@ -4169,7 +4170,7 @@
         <v>107</v>
       </c>
       <c r="AT11" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU11" t="s">
         <v>118</v>
@@ -4450,7 +4451,7 @@
         <v>107</v>
       </c>
       <c r="AT12" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU12" t="s">
         <v>118</v>
@@ -4740,7 +4741,7 @@
         <v>107</v>
       </c>
       <c r="AT13" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU13" t="s">
         <v>118</v>
@@ -5027,7 +5028,7 @@
         <v>107</v>
       </c>
       <c r="AT14" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU14" t="s">
         <v>118</v>
@@ -5305,7 +5306,7 @@
         <v>107</v>
       </c>
       <c r="AT15" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU15" t="s">
         <v>118</v>
@@ -5592,7 +5593,7 @@
         <v>111</v>
       </c>
       <c r="AT16" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU16" t="s">
         <v>118</v>
@@ -5882,7 +5883,7 @@
         <v>107</v>
       </c>
       <c r="AT17" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU17" t="s">
         <v>118</v>
@@ -6175,7 +6176,7 @@
         <v>107</v>
       </c>
       <c r="AT18" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="AU18" t="s">
         <v>118</v>
@@ -6462,7 +6463,7 @@
         <v>107</v>
       </c>
       <c r="AT19" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="AU19" t="s">
         <v>118</v>
@@ -6755,7 +6756,7 @@
         <v>111</v>
       </c>
       <c r="AT20" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU20" t="s">
         <v>118</v>
@@ -7042,7 +7043,7 @@
         <v>107</v>
       </c>
       <c r="AT21" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU21" t="s">
         <v>118</v>
@@ -7332,7 +7333,7 @@
         <v>107</v>
       </c>
       <c r="AT22" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="AU22" t="s">
         <v>118</v>
@@ -7619,7 +7620,7 @@
         <v>111</v>
       </c>
       <c r="AT23" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU23" t="s">
         <v>118</v>
@@ -7912,7 +7913,7 @@
         <v>107</v>
       </c>
       <c r="AT24" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU24" t="s">
         <v>118</v>
@@ -8205,7 +8206,7 @@
         <v>111</v>
       </c>
       <c r="AT25" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU25" t="s">
         <v>118</v>
@@ -8492,7 +8493,7 @@
         <v>107</v>
       </c>
       <c r="AT26" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU26" t="s">
         <v>118</v>
@@ -8779,7 +8780,7 @@
         <v>111</v>
       </c>
       <c r="AT27" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU27" t="s">
         <v>118</v>
@@ -9069,7 +9070,7 @@
         <v>107</v>
       </c>
       <c r="AT28" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU28" t="s">
         <v>118</v>
@@ -9362,7 +9363,7 @@
         <v>111</v>
       </c>
       <c r="AT29" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU29" t="s">
         <v>118</v>
@@ -9652,7 +9653,7 @@
         <v>111</v>
       </c>
       <c r="AT30" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU30" t="s">
         <v>118</v>
@@ -9942,7 +9943,7 @@
         <v>111</v>
       </c>
       <c r="AT31" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU31" t="s">
         <v>118</v>
@@ -10235,7 +10236,7 @@
         <v>111</v>
       </c>
       <c r="AT32" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU32" t="s">
         <v>118</v>
@@ -10519,7 +10520,7 @@
         <v>107</v>
       </c>
       <c r="AT33" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU33" t="s">
         <v>118</v>
@@ -10809,7 +10810,7 @@
         <v>111</v>
       </c>
       <c r="AT34" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU34" t="s">
         <v>118</v>
@@ -11102,7 +11103,7 @@
         <v>111</v>
       </c>
       <c r="AT35" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU35" t="s">
         <v>118</v>
@@ -11395,7 +11396,7 @@
         <v>111</v>
       </c>
       <c r="AT36" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU36" t="s">
         <v>118</v>
@@ -11679,7 +11680,7 @@
         <v>111</v>
       </c>
       <c r="AT37" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU37" t="s">
         <v>118</v>
@@ -11960,7 +11961,7 @@
         <v>107</v>
       </c>
       <c r="AT38" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU38" t="s">
         <v>118</v>
@@ -12244,7 +12245,7 @@
         <v>111</v>
       </c>
       <c r="AT39" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU39" t="s">
         <v>118</v>
@@ -12534,7 +12535,7 @@
         <v>111</v>
       </c>
       <c r="AT40" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU40" t="s">
         <v>118</v>
@@ -12818,7 +12819,7 @@
         <v>107</v>
       </c>
       <c r="AT41" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU41" t="s">
         <v>118</v>
@@ -13111,7 +13112,7 @@
         <v>111</v>
       </c>
       <c r="AT42" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU42" t="s">
         <v>118</v>
@@ -13395,13 +13396,13 @@
         <v>118</v>
       </c>
       <c r="AR43" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="AS43" t="s">
         <v>107</v>
       </c>
       <c r="AT43" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU43" t="s">
         <v>118</v>
@@ -13682,7 +13683,7 @@
         <v>111</v>
       </c>
       <c r="AT44" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU44" t="s">
         <v>118</v>
@@ -13975,7 +13976,7 @@
         <v>111</v>
       </c>
       <c r="AT45" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU45" t="s">
         <v>118</v>
@@ -14259,7 +14260,7 @@
         <v>107</v>
       </c>
       <c r="AT46" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU46" t="s">
         <v>118</v>
@@ -14546,7 +14547,7 @@
         <v>111</v>
       </c>
       <c r="AT47" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU47" t="s">
         <v>118</v>
@@ -14833,7 +14834,7 @@
         <v>111</v>
       </c>
       <c r="AT48" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU48" t="s">
         <v>118</v>
@@ -15129,7 +15130,7 @@
         <v>107</v>
       </c>
       <c r="AT49" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU49" t="s">
         <v>118</v>
@@ -15413,7 +15414,7 @@
         <v>111</v>
       </c>
       <c r="AT50" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU50" t="s">
         <v>118</v>
@@ -15712,7 +15713,7 @@
         <v>111</v>
       </c>
       <c r="AT51" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU51" t="s">
         <v>118</v>
@@ -16002,7 +16003,7 @@
         <v>111</v>
       </c>
       <c r="AT52" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU52" t="s">
         <v>105</v>
@@ -16295,7 +16296,7 @@
         <v>111</v>
       </c>
       <c r="AT53" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU53" t="s">
         <v>118</v>
@@ -16582,7 +16583,7 @@
         <v>107</v>
       </c>
       <c r="AT54" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU54" t="s">
         <v>118</v>
@@ -16869,7 +16870,7 @@
         <v>107</v>
       </c>
       <c r="AT55" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU55" t="s">
         <v>118</v>
@@ -17159,7 +17160,7 @@
         <v>111</v>
       </c>
       <c r="AT56" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU56" t="s">
         <v>118</v>
@@ -17452,7 +17453,7 @@
         <v>111</v>
       </c>
       <c r="AT57" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU57" t="s">
         <v>118</v>
@@ -17733,7 +17734,7 @@
         <v>111</v>
       </c>
       <c r="AT58" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU58" t="s">
         <v>118</v>
@@ -18029,7 +18030,7 @@
         <v>107</v>
       </c>
       <c r="AT59" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU59" t="s">
         <v>118</v>
@@ -18319,7 +18320,7 @@
         <v>111</v>
       </c>
       <c r="AT60" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU60" t="s">
         <v>118</v>
@@ -18618,7 +18619,7 @@
         <v>111</v>
       </c>
       <c r="AT61" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU61" t="s">
         <v>118</v>
@@ -18905,7 +18906,7 @@
         <v>107</v>
       </c>
       <c r="AT62" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU62" t="s">
         <v>118</v>
@@ -19201,7 +19202,7 @@
         <v>107</v>
       </c>
       <c r="AT63" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU63" t="s">
         <v>118</v>
@@ -19488,7 +19489,7 @@
         <v>111</v>
       </c>
       <c r="AT64" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU64" t="s">
         <v>118</v>
@@ -19775,7 +19776,7 @@
         <v>111</v>
       </c>
       <c r="AT65" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU65" t="s">
         <v>118</v>
@@ -20065,7 +20066,7 @@
         <v>111</v>
       </c>
       <c r="AT66" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU66" t="s">
         <v>118</v>
@@ -20349,7 +20350,7 @@
         <v>107</v>
       </c>
       <c r="AT67" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="AU67" t="s">
         <v>118</v>
@@ -20633,7 +20634,7 @@
         <v>107</v>
       </c>
       <c r="AT68" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU68" t="s">
         <v>118</v>
@@ -20923,7 +20924,7 @@
         <v>111</v>
       </c>
       <c r="AT69" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU69" t="s">
         <v>118</v>
@@ -21213,7 +21214,7 @@
         <v>111</v>
       </c>
       <c r="AT70" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="AU70" t="s">
         <v>118</v>
@@ -21512,7 +21513,7 @@
         <v>107</v>
       </c>
       <c r="AT71" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU71" t="s">
         <v>118</v>
@@ -21802,7 +21803,7 @@
         <v>111</v>
       </c>
       <c r="AT72" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU72" t="s">
         <v>118</v>
@@ -22092,7 +22093,7 @@
         <v>107</v>
       </c>
       <c r="AT73" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU73" t="s">
         <v>118</v>
@@ -22379,7 +22380,7 @@
         <v>107</v>
       </c>
       <c r="AT74" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU74" t="s">
         <v>118</v>
@@ -22678,7 +22679,7 @@
         <v>107</v>
       </c>
       <c r="AT75" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU75" t="s">
         <v>118</v>
@@ -22962,7 +22963,7 @@
         <v>111</v>
       </c>
       <c r="AT76" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU76" t="s">
         <v>118</v>
@@ -23252,7 +23253,7 @@
         <v>107</v>
       </c>
       <c r="AT77" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU77" t="s">
         <v>118</v>
@@ -23536,7 +23537,7 @@
         <v>111</v>
       </c>
       <c r="AT78" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU78" t="s">
         <v>118</v>
@@ -23832,7 +23833,7 @@
         <v>107</v>
       </c>
       <c r="AT79" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU79" t="s">
         <v>118</v>
@@ -24122,7 +24123,7 @@
         <v>107</v>
       </c>
       <c r="AT80" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU80" t="s">
         <v>118</v>
@@ -24406,7 +24407,7 @@
         <v>107</v>
       </c>
       <c r="AT81" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU81" t="s">
         <v>118</v>
@@ -24693,7 +24694,7 @@
         <v>111</v>
       </c>
       <c r="AT82" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU82" t="s">
         <v>118</v>
@@ -24986,7 +24987,7 @@
         <v>107</v>
       </c>
       <c r="AT83" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU83" t="s">
         <v>118</v>
@@ -25276,7 +25277,7 @@
         <v>111</v>
       </c>
       <c r="AT84" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU84" t="s">
         <v>118</v>
@@ -25566,7 +25567,7 @@
         <v>107</v>
       </c>
       <c r="AT85" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU85" t="s">
         <v>118</v>
@@ -25856,7 +25857,7 @@
         <v>107</v>
       </c>
       <c r="AT86" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="AU86" t="s">
         <v>118</v>
@@ -26146,7 +26147,7 @@
         <v>111</v>
       </c>
       <c r="AT87" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU87" t="s">
         <v>118</v>
@@ -26433,7 +26434,7 @@
         <v>107</v>
       </c>
       <c r="AT88" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU88" t="s">
         <v>118</v>
@@ -26723,7 +26724,7 @@
         <v>111</v>
       </c>
       <c r="AT89" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU89" t="s">
         <v>118</v>
@@ -27013,7 +27014,7 @@
         <v>107</v>
       </c>
       <c r="AT90" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU90" t="s">
         <v>118</v>
@@ -27306,7 +27307,7 @@
         <v>111</v>
       </c>
       <c r="AT91" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU91" t="s">
         <v>118</v>
@@ -27883,7 +27884,7 @@
         <v>111</v>
       </c>
       <c r="AT93" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU93" t="s">
         <v>118</v>
@@ -28176,7 +28177,7 @@
         <v>111</v>
       </c>
       <c r="AT94" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU94" t="s">
         <v>118</v>
@@ -28475,7 +28476,7 @@
         <v>111</v>
       </c>
       <c r="AT95" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU95" t="s">
         <v>118</v>
@@ -28765,7 +28766,7 @@
         <v>107</v>
       </c>
       <c r="AT96" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU96" t="s">
         <v>118</v>
@@ -29055,7 +29056,7 @@
         <v>111</v>
       </c>
       <c r="AT97" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU97" t="s">
         <v>118</v>
@@ -29348,7 +29349,7 @@
         <v>111</v>
       </c>
       <c r="AT98" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU98" t="s">
         <v>118</v>
@@ -29638,7 +29639,7 @@
         <v>111</v>
       </c>
       <c r="AT99" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU99" t="s">
         <v>118</v>
@@ -29937,7 +29938,7 @@
         <v>111</v>
       </c>
       <c r="AT100" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU100" t="s">
         <v>118</v>
@@ -30209,13 +30210,13 @@
         <v>1</v>
       </c>
       <c r="AR101" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="AS101" t="s">
         <v>111</v>
       </c>
       <c r="AT101" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU101" t="s">
         <v>118</v>
@@ -30502,7 +30503,7 @@
         <v>111</v>
       </c>
       <c r="AT102" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU102" t="s">
         <v>118</v>
@@ -30792,7 +30793,7 @@
         <v>111</v>
       </c>
       <c r="AT103" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU103" t="s">
         <v>118</v>
@@ -31369,7 +31370,7 @@
         <v>111</v>
       </c>
       <c r="AT105" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU105" t="s">
         <v>118</v>
@@ -31943,7 +31944,7 @@
         <v>111</v>
       </c>
       <c r="AT107" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU107" t="s">
         <v>111</v>
@@ -32230,7 +32231,7 @@
         <v>111</v>
       </c>
       <c r="AT108" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU108" t="s">
         <v>118</v>
@@ -32517,7 +32518,7 @@
         <v>111</v>
       </c>
       <c r="AT109" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU109" t="s">
         <v>118</v>
@@ -32804,7 +32805,7 @@
         <v>107</v>
       </c>
       <c r="AT110" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU110" t="s">
         <v>118</v>
@@ -33091,7 +33092,7 @@
         <v>111</v>
       </c>
       <c r="AT111" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU111" t="s">
         <v>118</v>
@@ -33378,7 +33379,7 @@
         <v>111</v>
       </c>
       <c r="AT112" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU112" t="s">
         <v>118</v>
@@ -33668,7 +33669,7 @@
         <v>107</v>
       </c>
       <c r="AT113" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU113" t="s">
         <v>118</v>
@@ -33961,7 +33962,7 @@
         <v>111</v>
       </c>
       <c r="AT114" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU114" t="s">
         <v>118</v>
@@ -34248,7 +34249,7 @@
         <v>111</v>
       </c>
       <c r="AT115" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU115" t="s">
         <v>118</v>
@@ -34541,7 +34542,7 @@
         <v>111</v>
       </c>
       <c r="AT116" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU116" t="s">
         <v>118</v>
@@ -34822,7 +34823,7 @@
         <v>111</v>
       </c>
       <c r="AT117" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU117" t="s">
         <v>118</v>
@@ -35106,7 +35107,7 @@
         <v>111</v>
       </c>
       <c r="AT118" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU118" t="s">
         <v>118</v>
@@ -35393,7 +35394,7 @@
         <v>111</v>
       </c>
       <c r="AT119" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="AU119" t="s">
         <v>118</v>
@@ -35683,7 +35684,7 @@
         <v>111</v>
       </c>
       <c r="AT120" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU120" t="s">
         <v>118</v>
@@ -35967,7 +35968,7 @@
         <v>111</v>
       </c>
       <c r="AT121" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU121" t="s">
         <v>118</v>
@@ -36544,7 +36545,7 @@
         <v>111</v>
       </c>
       <c r="AT123" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="AU123" t="s">
         <v>118</v>
@@ -36831,7 +36832,7 @@
         <v>111</v>
       </c>
       <c r="AT124" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU124" t="s">
         <v>118</v>
@@ -37695,7 +37696,7 @@
         <v>111</v>
       </c>
       <c r="AT127" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU127" t="s">
         <v>118</v>
@@ -37982,7 +37983,7 @@
         <v>111</v>
       </c>
       <c r="AT128" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU128" t="s">
         <v>118</v>
@@ -38568,7 +38569,7 @@
         <v>107</v>
       </c>
       <c r="AT130" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="AU130" t="s">
         <v>118</v>
@@ -38855,7 +38856,7 @@
         <v>111</v>
       </c>
       <c r="AT131" t="s">
-        <v>137</v>
+        <v>262</v>
       </c>
       <c r="AU131" t="s">
         <v>118</v>
@@ -39429,7 +39430,7 @@
         <v>107</v>
       </c>
       <c r="AT133" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU133" t="s">
         <v>118</v>
@@ -39716,7 +39717,7 @@
         <v>111</v>
       </c>
       <c r="AT134" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU134" t="s">
         <v>118</v>
@@ -40006,7 +40007,7 @@
         <v>107</v>
       </c>
       <c r="AT135" t="s">
-        <v>263</v>
+        <v>137</v>
       </c>
       <c r="AU135" t="s">
         <v>118</v>
@@ -40293,7 +40294,7 @@
         <v>107</v>
       </c>
       <c r="AT136" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="AU136" t="s">
         <v>118</v>

</xml_diff>